<commit_message>
data fill, draw ER
</commit_message>
<xml_diff>
--- a/documentation.xlsx
+++ b/documentation.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java eCube\Full Stack Course\classes\Ei Yadanar\java\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{584F661D-FBE1-4910-9D76-C24693591E7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2D8A35B1-B1F6-41D8-9AD1-C151D75ED4D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{D5483A6E-828E-4639-B2BD-0469AAAA7367}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{D5483A6E-828E-4639-B2BD-0469AAAA7367}"/>
   </bookViews>
   <sheets>
     <sheet name="requirement" sheetId="1" r:id="rId1"/>
     <sheet name="usecase" sheetId="2" r:id="rId2"/>
     <sheet name="raw material" sheetId="3" r:id="rId3"/>
+    <sheet name="database" sheetId="4" r:id="rId4"/>
+    <sheet name="ER" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="72">
   <si>
     <t>requirements</t>
   </si>
@@ -80,18 +82,225 @@
   </si>
   <si>
     <t>main drink</t>
+  </si>
+  <si>
+    <t>brownsugar milk</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>brownsugar chese milk</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>milktea(redtea,uron tea,jasmine tea)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>tea(redtea,uron tea,jasmine tea)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mango juice(with milk)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>orange tea(with jasmine tea)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>kiwi juice</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>mango tea(with jasmine tea)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>topping</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>bubble</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>coconut jelly</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>gress jelly(taiwan jelly)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>chese</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>ice(max,less,no-&gt;(+\50))</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>sugar level(100%,70%(normal),50%,30%,0%)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>tea</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>juice</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>brown sugar</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>orange,kiwi,mango,tea,milk</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>macha,red,uron,jasmine,milk,brown sugar</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>brownsugar milktea(red tea,uron tea,jasmine tea,macha)</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>cheese</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>brown sugar milk</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>c_id</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>macha</t>
+  </si>
+  <si>
+    <t>red</t>
+  </si>
+  <si>
+    <t>uron</t>
+  </si>
+  <si>
+    <t>jasmine</t>
+  </si>
+  <si>
+    <t>milk</t>
+  </si>
+  <si>
+    <t>brown sugar</t>
+  </si>
+  <si>
+    <t>orange</t>
+  </si>
+  <si>
+    <t>kiwi</t>
+  </si>
+  <si>
+    <t>mango</t>
+  </si>
+  <si>
+    <t>tea</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>catetory</t>
+  </si>
+  <si>
+    <t>Topping</t>
+  </si>
+  <si>
+    <t>t_id</t>
+  </si>
+  <si>
+    <t>kinds</t>
+  </si>
+  <si>
+    <t>Order</t>
+  </si>
+  <si>
+    <t>m_id</t>
+  </si>
+  <si>
+    <t>1,3</t>
+  </si>
+  <si>
+    <t>Ice</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Less</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>SugerLevel</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Size</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>i_id</t>
+  </si>
+  <si>
+    <t>s_id</t>
+  </si>
+  <si>
+    <t>amount</t>
+  </si>
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>order_id</t>
+  </si>
+  <si>
+    <t>Ture</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="6"/>
+      <name val="Aptos Narrow"/>
+      <family val="3"/>
+      <charset val="128"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -103,7 +312,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -111,13 +320,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2487,6 +2714,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2505,6 +2733,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -2512,15 +2741,565 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FA4C0CB-15B5-4D2F-B3B4-F56002FD090E}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>12</v>
+      </c>
+      <c r="G1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="G2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A917FDAE-9AEC-416A-A094-3DCBFC4E0305}">
+  <dimension ref="A1:O21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.77734375" customWidth="1"/>
+    <col min="7" max="7" width="9.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I1" t="s">
+        <v>57</v>
+      </c>
+      <c r="M1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="2">
+        <v>1</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="2">
+        <v>1</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="K3" s="2">
+        <v>50</v>
+      </c>
+      <c r="M3" s="2">
+        <v>1</v>
+      </c>
+      <c r="N3" s="2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="2">
+        <v>2</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="2">
+        <v>2</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="K4" s="2">
+        <v>0</v>
+      </c>
+      <c r="M4" s="2">
+        <v>2</v>
+      </c>
+      <c r="N4" s="2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="2">
+        <v>3</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I5" s="2">
+        <v>3</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="K5" s="2">
+        <v>0</v>
+      </c>
+      <c r="M5" s="2">
+        <v>3</v>
+      </c>
+      <c r="N5" s="2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="E6" s="2">
+        <v>4</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="M6" s="2">
+        <v>4</v>
+      </c>
+      <c r="N6" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="M7" s="2">
+        <v>5</v>
+      </c>
+      <c r="N7" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A10" s="2">
+        <v>1</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="2">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2">
+        <v>650</v>
+      </c>
+      <c r="G10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A11" s="2">
+        <v>2</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="2">
+        <v>1</v>
+      </c>
+      <c r="D11" s="2">
+        <v>700</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="O11" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A12" s="2">
+        <v>3</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="2">
+        <v>1</v>
+      </c>
+      <c r="D12" s="2">
+        <v>400</v>
+      </c>
+      <c r="G12" s="4">
+        <v>46199</v>
+      </c>
+      <c r="H12" s="2">
+        <v>1</v>
+      </c>
+      <c r="I12" s="2">
+        <v>1</v>
+      </c>
+      <c r="J12" s="2">
+        <v>2</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="L12" s="2">
+        <v>1</v>
+      </c>
+      <c r="M12" s="2">
+        <v>4</v>
+      </c>
+      <c r="N12" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O12" s="2">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A13" s="2">
+        <v>4</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="2">
+        <v>1</v>
+      </c>
+      <c r="D13" s="3">
+        <v>333.33333333333297</v>
+      </c>
+      <c r="G13" s="4">
+        <v>46199</v>
+      </c>
+      <c r="H13" s="2">
+        <v>2</v>
+      </c>
+      <c r="I13" s="2">
+        <v>1</v>
+      </c>
+      <c r="J13" s="2">
+        <v>1</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="L13" s="2">
+        <v>1</v>
+      </c>
+      <c r="M13" s="2">
+        <v>4</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="O13" s="2"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A14" s="2">
+        <v>5</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="2">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A15" s="2">
+        <v>6</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="2">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3">
+        <v>644.444444444444</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A16" s="2">
+        <v>7</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="2">
+        <v>2</v>
+      </c>
+      <c r="D16" s="3">
+        <v>744.444444444444</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="2">
+        <v>8</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="2">
+        <v>3</v>
+      </c>
+      <c r="D17" s="3">
+        <v>844.444444444444</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="2">
+        <v>9</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" s="2">
+        <v>3</v>
+      </c>
+      <c r="D18" s="3">
+        <v>944.444444444444</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="2">
+        <v>10</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C19" s="2">
+        <v>3</v>
+      </c>
+      <c r="D19" s="3">
+        <v>1044.44444444444</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="2">
+        <v>11</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20" s="2">
+        <v>3</v>
+      </c>
+      <c r="D20" s="3">
+        <v>1144.44444444444</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="2">
+        <v>12</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" s="2">
+        <v>3</v>
+      </c>
+      <c r="D21" s="3">
+        <v>1244.44444444444</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF7CD0A0-FCF4-4193-A804-F8D42B1C7605}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>